<commit_message>
HU wind bids: one set of key dates for all projects
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Cy4jTfjKbxPfMRQvaZwVT
</commit_message>
<xml_diff>
--- a/projects/hu_wind_2/out/HU_Wind_bids.xlsx
+++ b/projects/hu_wind_2/out/HU_Wind_bids.xlsx
@@ -18,6 +18,15 @@
     <definedName name="PB_Rate">Inputs!$E$10</definedName>
     <definedName name="Part_Fee">Inputs!$E$11</definedName>
     <definedName name="TSO_Rate">Inputs!$E$12</definedName>
+    <definedName name="Date_Sign">Inputs!$E$27</definedName>
+    <definedName name="Date_Bid">Inputs!$E$28</definedName>
+    <definedName name="Date_PB">Inputs!$E$29</definedName>
+    <definedName name="Date_TSO">Inputs!$E$30</definedName>
+    <definedName name="Date_Devex">Inputs!$E$31</definedName>
+    <definedName name="Date_HC">Inputs!$E$32</definedName>
+    <definedName name="Date_NTP">Inputs!$E$33</definedName>
+    <definedName name="Date_COD">Inputs!$E$34</definedName>
+    <definedName name="Date_Release">Inputs!$E$35</definedName>
     <definedName name="Rate_Cash">Inputs!$E$37</definedName>
     <definedName name="Rate_Devex">Inputs!$E$38</definedName>
     <definedName name="Devex_Floor">Inputs!$E$39</definedName>
@@ -1755,17 +1764,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Date: Bora</t>
-        </is>
-      </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>Iváncsa</t>
-        </is>
-      </c>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>Dunaújváros</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
@@ -1797,15 +1796,7 @@
         <v/>
       </c>
       <c r="J47" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K47" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L47" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -1837,15 +1828,7 @@
         <v/>
       </c>
       <c r="J48" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K48" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L48" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -1877,15 +1860,7 @@
         <v/>
       </c>
       <c r="J49" s="18">
-        <f>Inputs!E$28</f>
-        <v/>
-      </c>
-      <c r="K49" s="18">
-        <f>Inputs!F$28</f>
-        <v/>
-      </c>
-      <c r="L49" s="18">
-        <f>Inputs!G$28</f>
+        <f>Date_PB</f>
         <v/>
       </c>
     </row>
@@ -1945,15 +1920,7 @@
         <v/>
       </c>
       <c r="J51" s="18">
-        <f>Inputs!E$28</f>
-        <v/>
-      </c>
-      <c r="K51" s="18">
-        <f>Inputs!F$28</f>
-        <v/>
-      </c>
-      <c r="L51" s="18">
-        <f>Inputs!G$28</f>
+        <f>Date_PB</f>
         <v/>
       </c>
     </row>
@@ -1985,15 +1952,7 @@
         <v/>
       </c>
       <c r="J52" s="18">
-        <f>Inputs!E$29</f>
-        <v/>
-      </c>
-      <c r="K52" s="18">
-        <f>Inputs!F$29</f>
-        <v/>
-      </c>
-      <c r="L52" s="18">
-        <f>Inputs!G$29</f>
+        <f>Date_TSO</f>
         <v/>
       </c>
     </row>
@@ -2025,15 +1984,7 @@
         <v/>
       </c>
       <c r="J53" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K53" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L53" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -2065,15 +2016,7 @@
         <v/>
       </c>
       <c r="J54" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K54" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L54" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -2133,15 +2076,7 @@
         <v/>
       </c>
       <c r="J56" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K56" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L56" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -2173,15 +2108,7 @@
         <v/>
       </c>
       <c r="J57" s="18">
-        <f>Inputs!E$31</f>
-        <v/>
-      </c>
-      <c r="K57" s="18">
-        <f>Inputs!F$31</f>
-        <v/>
-      </c>
-      <c r="L57" s="18">
-        <f>Inputs!G$31</f>
+        <f>Date_Devex</f>
         <v/>
       </c>
     </row>
@@ -2247,17 +2174,7 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Date: Bora</t>
-        </is>
-      </c>
-      <c r="K60" s="5" t="inlineStr">
-        <is>
-          <t>Iváncsa</t>
-        </is>
-      </c>
-      <c r="L60" s="5" t="inlineStr">
-        <is>
-          <t>Dunaújváros</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
@@ -2289,15 +2206,7 @@
         <v/>
       </c>
       <c r="J61" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K61" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L61" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -2329,15 +2238,7 @@
         <v/>
       </c>
       <c r="J62" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K62" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L62" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -2369,15 +2270,7 @@
         <v/>
       </c>
       <c r="J63" s="18">
-        <f>Inputs!E$28</f>
-        <v/>
-      </c>
-      <c r="K63" s="18">
-        <f>Inputs!F$28</f>
-        <v/>
-      </c>
-      <c r="L63" s="18">
-        <f>Inputs!G$28</f>
+        <f>Date_PB</f>
         <v/>
       </c>
     </row>
@@ -2409,15 +2302,7 @@
         <v/>
       </c>
       <c r="J64" s="18">
-        <f>Inputs!E$29</f>
-        <v/>
-      </c>
-      <c r="K64" s="18">
-        <f>Inputs!F$29</f>
-        <v/>
-      </c>
-      <c r="L64" s="18">
-        <f>Inputs!G$29</f>
+        <f>Date_TSO</f>
         <v/>
       </c>
     </row>
@@ -2449,15 +2334,7 @@
         <v/>
       </c>
       <c r="J65" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K65" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L65" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -2489,15 +2366,7 @@
         <v/>
       </c>
       <c r="J66" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K66" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L66" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -2529,15 +2398,7 @@
         <v/>
       </c>
       <c r="J67" s="18">
-        <f>Inputs!E$31</f>
-        <v/>
-      </c>
-      <c r="K67" s="18">
-        <f>Inputs!F$31</f>
-        <v/>
-      </c>
-      <c r="L67" s="18">
-        <f>Inputs!G$31</f>
+        <f>Date_Devex</f>
         <v/>
       </c>
     </row>
@@ -2569,15 +2430,7 @@
         <v/>
       </c>
       <c r="J68" s="18">
-        <f>Inputs!E$26</f>
-        <v/>
-      </c>
-      <c r="K68" s="18">
-        <f>Inputs!F$26</f>
-        <v/>
-      </c>
-      <c r="L68" s="18">
-        <f>Inputs!G$26</f>
+        <f>Date_Sign</f>
         <v/>
       </c>
     </row>
@@ -3576,11 +3429,11 @@
         <v/>
       </c>
       <c r="F107" s="23">
-        <f>XIRR(F190:F198,K190:K198)</f>
+        <f>XIRR(F190:F198,J190:J198)</f>
         <v/>
       </c>
       <c r="G107" s="23">
-        <f>XIRR(G190:G198,L190:L198)</f>
+        <f>XIRR(G190:G198,J190:J198)</f>
         <v/>
       </c>
     </row>
@@ -7308,15 +7161,15 @@
         </is>
       </c>
       <c r="E156" s="27">
-        <f>DATE(YEAR(Inputs!E$27)+1,1,1)-Inputs!E$27</f>
+        <f>DATE(YEAR(Date_Bid)+1,1,1)-Date_Bid</f>
         <v/>
       </c>
       <c r="F156" s="27">
-        <f>DATE(YEAR(Inputs!F$27)+1,1,1)-Inputs!F$27</f>
+        <f>DATE(YEAR(Date_Bid)+1,1,1)-Date_Bid</f>
         <v/>
       </c>
       <c r="G156" s="27">
-        <f>DATE(YEAR(Inputs!G$27)+1,1,1)-Inputs!G$27</f>
+        <f>DATE(YEAR(Date_Bid)+1,1,1)-Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -7332,15 +7185,15 @@
         </is>
       </c>
       <c r="E157" s="26">
-        <f>(1+Rate_Cash*E156/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Inputs!E$27)-1)*E154</f>
+        <f>(1+Rate_Cash*E156/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Date_Bid)-1)*E154</f>
         <v/>
       </c>
       <c r="F157" s="26">
-        <f>(1+Rate_Cash*F156/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Inputs!F$27)-1)*F154</f>
+        <f>(1+Rate_Cash*F156/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Date_Bid)-1)*F154</f>
         <v/>
       </c>
       <c r="G157" s="26">
-        <f>(1+Rate_Cash*G156/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Inputs!G$27)-1)*G154</f>
+        <f>(1+Rate_Cash*G156/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Date_Bid)-1)*G154</f>
         <v/>
       </c>
     </row>
@@ -7356,15 +7209,15 @@
         </is>
       </c>
       <c r="E158" s="27">
-        <f>DATE(YEAR(Inputs!E$28)+1,1,1)-Inputs!E$28</f>
+        <f>DATE(YEAR(Date_PB)+1,1,1)-Date_PB</f>
         <v/>
       </c>
       <c r="F158" s="27">
-        <f>DATE(YEAR(Inputs!F$28)+1,1,1)-Inputs!F$28</f>
+        <f>DATE(YEAR(Date_PB)+1,1,1)-Date_PB</f>
         <v/>
       </c>
       <c r="G158" s="27">
-        <f>DATE(YEAR(Inputs!G$28)+1,1,1)-Inputs!G$28</f>
+        <f>DATE(YEAR(Date_PB)+1,1,1)-Date_PB</f>
         <v/>
       </c>
     </row>
@@ -7380,15 +7233,15 @@
         </is>
       </c>
       <c r="E159" s="26">
-        <f>(1+Rate_Cash*E158/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Inputs!E$28)-1)*E154</f>
+        <f>(1+Rate_Cash*E158/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Date_PB)-1)*E154</f>
         <v/>
       </c>
       <c r="F159" s="26">
-        <f>(1+Rate_Cash*F158/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Inputs!F$28)-1)*F154</f>
+        <f>(1+Rate_Cash*F158/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Date_PB)-1)*F154</f>
         <v/>
       </c>
       <c r="G159" s="26">
-        <f>(1+Rate_Cash*G158/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Inputs!G$28)-1)*G154</f>
+        <f>(1+Rate_Cash*G158/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Date_PB)-1)*G154</f>
         <v/>
       </c>
     </row>
@@ -7404,15 +7257,15 @@
         </is>
       </c>
       <c r="E160" s="27">
-        <f>DATE(YEAR(Inputs!E$29)+1,1,1)-Inputs!E$29</f>
+        <f>DATE(YEAR(Date_TSO)+1,1,1)-Date_TSO</f>
         <v/>
       </c>
       <c r="F160" s="27">
-        <f>DATE(YEAR(Inputs!F$29)+1,1,1)-Inputs!F$29</f>
+        <f>DATE(YEAR(Date_TSO)+1,1,1)-Date_TSO</f>
         <v/>
       </c>
       <c r="G160" s="27">
-        <f>DATE(YEAR(Inputs!G$29)+1,1,1)-Inputs!G$29</f>
+        <f>DATE(YEAR(Date_TSO)+1,1,1)-Date_TSO</f>
         <v/>
       </c>
     </row>
@@ -7428,15 +7281,15 @@
         </is>
       </c>
       <c r="E161" s="26">
-        <f>(1+Rate_Cash*E160/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Inputs!E$29)-1)*E154</f>
+        <f>(1+Rate_Cash*E160/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Date_TSO)-1)*E154</f>
         <v/>
       </c>
       <c r="F161" s="26">
-        <f>(1+Rate_Cash*F160/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Inputs!F$29)-1)*F154</f>
+        <f>(1+Rate_Cash*F160/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Date_TSO)-1)*F154</f>
         <v/>
       </c>
       <c r="G161" s="26">
-        <f>(1+Rate_Cash*G160/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Inputs!G$29)-1)*G154</f>
+        <f>(1+Rate_Cash*G160/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Date_TSO)-1)*G154</f>
         <v/>
       </c>
     </row>
@@ -7452,15 +7305,15 @@
         </is>
       </c>
       <c r="E162" s="27">
-        <f>DATE(YEAR(Inputs!E$30)+1,1,1)-Inputs!E$30</f>
+        <f>DATE(YEAR(Date_HC)+1,1,1)-Date_HC</f>
         <v/>
       </c>
       <c r="F162" s="27">
-        <f>DATE(YEAR(Inputs!F$30)+1,1,1)-Inputs!F$30</f>
+        <f>DATE(YEAR(Date_HC)+1,1,1)-Date_HC</f>
         <v/>
       </c>
       <c r="G162" s="27">
-        <f>DATE(YEAR(Inputs!G$30)+1,1,1)-Inputs!G$30</f>
+        <f>DATE(YEAR(Date_HC)+1,1,1)-Date_HC</f>
         <v/>
       </c>
     </row>
@@ -7476,15 +7329,15 @@
         </is>
       </c>
       <c r="E163" s="26">
-        <f>(1+Rate_Cash*E162/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Inputs!E$30)-1)*E154</f>
+        <f>(1+Rate_Cash*E162/Days_In_Year)*(1+Rate_Cash)^(YEAR(E153)-YEAR(Date_HC)-1)*E154</f>
         <v/>
       </c>
       <c r="F163" s="26">
-        <f>(1+Rate_Cash*F162/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Inputs!F$30)-1)*F154</f>
+        <f>(1+Rate_Cash*F162/Days_In_Year)*(1+Rate_Cash)^(YEAR(F153)-YEAR(Date_HC)-1)*F154</f>
         <v/>
       </c>
       <c r="G163" s="26">
-        <f>(1+Rate_Cash*G162/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Inputs!G$30)-1)*G154</f>
+        <f>(1+Rate_Cash*G162/Days_In_Year)*(1+Rate_Cash)^(YEAR(G153)-YEAR(Date_HC)-1)*G154</f>
         <v/>
       </c>
     </row>
@@ -7500,15 +7353,15 @@
         </is>
       </c>
       <c r="E164" s="27">
-        <f>DATE(YEAR(Inputs!E$31)+1,1,1)-Inputs!E$31</f>
+        <f>DATE(YEAR(Date_Devex)+1,1,1)-Date_Devex</f>
         <v/>
       </c>
       <c r="F164" s="27">
-        <f>DATE(YEAR(Inputs!F$31)+1,1,1)-Inputs!F$31</f>
+        <f>DATE(YEAR(Date_Devex)+1,1,1)-Date_Devex</f>
         <v/>
       </c>
       <c r="G164" s="27">
-        <f>DATE(YEAR(Inputs!G$31)+1,1,1)-Inputs!G$31</f>
+        <f>DATE(YEAR(Date_Devex)+1,1,1)-Date_Devex</f>
         <v/>
       </c>
     </row>
@@ -7524,15 +7377,15 @@
         </is>
       </c>
       <c r="E165" s="26">
-        <f>(1+Rate_Devex*E164/Days_In_Year)*(1+Rate_Devex)^(YEAR(E153)-YEAR(Inputs!E$31)-1)*E155</f>
+        <f>(1+Rate_Devex*E164/Days_In_Year)*(1+Rate_Devex)^(YEAR(E153)-YEAR(Date_Devex)-1)*E155</f>
         <v/>
       </c>
       <c r="F165" s="26">
-        <f>(1+Rate_Devex*F164/Days_In_Year)*(1+Rate_Devex)^(YEAR(F153)-YEAR(Inputs!F$31)-1)*F155</f>
+        <f>(1+Rate_Devex*F164/Days_In_Year)*(1+Rate_Devex)^(YEAR(F153)-YEAR(Date_Devex)-1)*F155</f>
         <v/>
       </c>
       <c r="G165" s="26">
-        <f>(1+Rate_Devex*G164/Days_In_Year)*(1+Rate_Devex)^(YEAR(G153)-YEAR(Inputs!G$31)-1)*G155</f>
+        <f>(1+Rate_Devex*G164/Days_In_Year)*(1+Rate_Devex)^(YEAR(G153)-YEAR(Date_Devex)-1)*G155</f>
         <v/>
       </c>
     </row>
@@ -7772,15 +7625,15 @@
         </is>
       </c>
       <c r="E174" s="8">
-        <f>E20*MIN(DSA_Rate*YEARFRAC(Inputs!E$35,Sale_Date),DSA_Cap)*E42</f>
+        <f>E20*MIN(DSA_Rate*YEARFRAC(Date_Sign,Sale_Date),DSA_Cap)*E42</f>
         <v/>
       </c>
       <c r="F174" s="8">
-        <f>F20*MIN(DSA_Rate*YEARFRAC(Inputs!F$35,Sale_Date),DSA_Cap)*F42</f>
+        <f>F20*MIN(DSA_Rate*YEARFRAC(Date_Sign,Sale_Date),DSA_Cap)*F42</f>
         <v/>
       </c>
       <c r="G174" s="8">
-        <f>G20*MIN(DSA_Rate*YEARFRAC(Inputs!G$35,Sale_Date),DSA_Cap)*G42</f>
+        <f>G20*MIN(DSA_Rate*YEARFRAC(Date_Sign,Sale_Date),DSA_Cap)*G42</f>
         <v/>
       </c>
       <c r="H174" s="8">
@@ -8160,17 +8013,7 @@
       </c>
       <c r="J189" s="21" t="inlineStr">
         <is>
-          <t>Date: Bora</t>
-        </is>
-      </c>
-      <c r="K189" s="21" t="inlineStr">
-        <is>
-          <t>Iváncsa</t>
-        </is>
-      </c>
-      <c r="L189" s="21" t="inlineStr">
-        <is>
-          <t>Dunaújváros</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
@@ -8202,15 +8045,7 @@
         <v/>
       </c>
       <c r="J190" s="18">
-        <f>Inputs!E$26</f>
-        <v/>
-      </c>
-      <c r="K190" s="18">
-        <f>Inputs!F$26</f>
-        <v/>
-      </c>
-      <c r="L190" s="18">
-        <f>Inputs!G$26</f>
+        <f>Date_Sign</f>
         <v/>
       </c>
     </row>
@@ -8242,15 +8077,7 @@
         <v/>
       </c>
       <c r="J191" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K191" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L191" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -8282,15 +8109,7 @@
         <v/>
       </c>
       <c r="J192" s="18">
-        <f>Inputs!E$27</f>
-        <v/>
-      </c>
-      <c r="K192" s="18">
-        <f>Inputs!F$27</f>
-        <v/>
-      </c>
-      <c r="L192" s="18">
-        <f>Inputs!G$27</f>
+        <f>Date_Bid</f>
         <v/>
       </c>
     </row>
@@ -8322,15 +8141,7 @@
         <v/>
       </c>
       <c r="J193" s="18">
-        <f>Inputs!E$28</f>
-        <v/>
-      </c>
-      <c r="K193" s="18">
-        <f>Inputs!F$28</f>
-        <v/>
-      </c>
-      <c r="L193" s="18">
-        <f>Inputs!G$28</f>
+        <f>Date_PB</f>
         <v/>
       </c>
     </row>
@@ -8362,15 +8173,7 @@
         <v/>
       </c>
       <c r="J194" s="18">
-        <f>Inputs!E$29</f>
-        <v/>
-      </c>
-      <c r="K194" s="18">
-        <f>Inputs!F$29</f>
-        <v/>
-      </c>
-      <c r="L194" s="18">
-        <f>Inputs!G$29</f>
+        <f>Date_TSO</f>
         <v/>
       </c>
     </row>
@@ -8402,15 +8205,7 @@
         <v/>
       </c>
       <c r="J195" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K195" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L195" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -8442,15 +8237,7 @@
         <v/>
       </c>
       <c r="J196" s="18">
-        <f>Inputs!E$30</f>
-        <v/>
-      </c>
-      <c r="K196" s="18">
-        <f>Inputs!F$30</f>
-        <v/>
-      </c>
-      <c r="L196" s="18">
-        <f>Inputs!G$30</f>
+        <f>Date_HC</f>
         <v/>
       </c>
     </row>
@@ -8482,15 +8269,7 @@
         <v/>
       </c>
       <c r="J197" s="18">
-        <f>Inputs!E$31</f>
-        <v/>
-      </c>
-      <c r="K197" s="18">
-        <f>Inputs!F$31</f>
-        <v/>
-      </c>
-      <c r="L197" s="18">
-        <f>Inputs!G$31</f>
+        <f>Date_Devex</f>
         <v/>
       </c>
     </row>
@@ -8522,14 +8301,6 @@
         <v/>
       </c>
       <c r="J198" s="18">
-        <f>Sale_Date</f>
-        <v/>
-      </c>
-      <c r="K198" s="18">
-        <f>Sale_Date</f>
-        <v/>
-      </c>
-      <c r="L198" s="18">
         <f>Sale_Date</f>
         <v/>
       </c>
@@ -9062,147 +8833,147 @@
         </is>
       </c>
       <c r="J208" s="27">
-        <f>J$204-YEAR(Inputs!$E$33)</f>
+        <f>J$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="K208" s="27">
-        <f>K$204-YEAR(Inputs!$E$33)</f>
+        <f>K$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="L208" s="27">
-        <f>L$204-YEAR(Inputs!$E$33)</f>
+        <f>L$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="M208" s="27">
-        <f>M$204-YEAR(Inputs!$E$33)</f>
+        <f>M$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="N208" s="27">
-        <f>N$204-YEAR(Inputs!$E$33)</f>
+        <f>N$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="O208" s="27">
-        <f>O$204-YEAR(Inputs!$E$33)</f>
+        <f>O$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="P208" s="27">
-        <f>P$204-YEAR(Inputs!$E$33)</f>
+        <f>P$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Q208" s="27">
-        <f>Q$204-YEAR(Inputs!$E$33)</f>
+        <f>Q$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="R208" s="27">
-        <f>R$204-YEAR(Inputs!$E$33)</f>
+        <f>R$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="S208" s="27">
-        <f>S$204-YEAR(Inputs!$E$33)</f>
+        <f>S$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="T208" s="27">
-        <f>T$204-YEAR(Inputs!$E$33)</f>
+        <f>T$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="U208" s="27">
-        <f>U$204-YEAR(Inputs!$E$33)</f>
+        <f>U$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="V208" s="27">
-        <f>V$204-YEAR(Inputs!$E$33)</f>
+        <f>V$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="W208" s="27">
-        <f>W$204-YEAR(Inputs!$E$33)</f>
+        <f>W$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="X208" s="27">
-        <f>X$204-YEAR(Inputs!$E$33)</f>
+        <f>X$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Y208" s="27">
-        <f>Y$204-YEAR(Inputs!$E$33)</f>
+        <f>Y$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Z208" s="27">
-        <f>Z$204-YEAR(Inputs!$E$33)</f>
+        <f>Z$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AA208" s="27">
-        <f>AA$204-YEAR(Inputs!$E$33)</f>
+        <f>AA$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AB208" s="27">
-        <f>AB$204-YEAR(Inputs!$E$33)</f>
+        <f>AB$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AC208" s="27">
-        <f>AC$204-YEAR(Inputs!$E$33)</f>
+        <f>AC$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AD208" s="27">
-        <f>AD$204-YEAR(Inputs!$E$33)</f>
+        <f>AD$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AE208" s="27">
-        <f>AE$204-YEAR(Inputs!$E$33)</f>
+        <f>AE$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AF208" s="27">
-        <f>AF$204-YEAR(Inputs!$E$33)</f>
+        <f>AF$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AG208" s="27">
-        <f>AG$204-YEAR(Inputs!$E$33)</f>
+        <f>AG$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AH208" s="27">
-        <f>AH$204-YEAR(Inputs!$E$33)</f>
+        <f>AH$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AI208" s="27">
-        <f>AI$204-YEAR(Inputs!$E$33)</f>
+        <f>AI$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ208" s="27">
-        <f>AJ$204-YEAR(Inputs!$E$33)</f>
+        <f>AJ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AK208" s="27">
-        <f>AK$204-YEAR(Inputs!$E$33)</f>
+        <f>AK$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AL208" s="27">
-        <f>AL$204-YEAR(Inputs!$E$33)</f>
+        <f>AL$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AM208" s="27">
-        <f>AM$204-YEAR(Inputs!$E$33)</f>
+        <f>AM$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AN208" s="27">
-        <f>AN$204-YEAR(Inputs!$E$33)</f>
+        <f>AN$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AO208" s="27">
-        <f>AO$204-YEAR(Inputs!$E$33)</f>
+        <f>AO$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AP208" s="27">
-        <f>AP$204-YEAR(Inputs!$E$33)</f>
+        <f>AP$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ208" s="27">
-        <f>AQ$204-YEAR(Inputs!$E$33)</f>
+        <f>AQ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AR208" s="27">
-        <f>AR$204-YEAR(Inputs!$E$33)</f>
+        <f>AR$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AS208" s="27">
-        <f>AS$204-YEAR(Inputs!$E$33)</f>
+        <f>AS$204-YEAR(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -9218,151 +8989,151 @@
         </is>
       </c>
       <c r="E209" s="27">
-        <f>DATEDIF(Inputs!$E$32,Inputs!$E$33,"m")</f>
+        <f>DATEDIF(Date_NTP,Date_COD,"m")</f>
         <v/>
       </c>
       <c r="J209" s="27">
-        <f>(J$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(J$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="K209" s="27">
-        <f>(K$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(K$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="L209" s="27">
-        <f>(L$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(L$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="M209" s="27">
-        <f>(M$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(M$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="N209" s="27">
-        <f>(N$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(N$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="O209" s="27">
-        <f>(O$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(O$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="P209" s="27">
-        <f>(P$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(P$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Q209" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(Q$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="R209" s="27">
-        <f>(R$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(R$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="S209" s="27">
-        <f>(S$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(S$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="T209" s="27">
-        <f>(T$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(T$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="U209" s="27">
-        <f>(U$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(U$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="V209" s="27">
-        <f>(V$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(V$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="W209" s="27">
-        <f>(W$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(W$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="X209" s="27">
-        <f>(X$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(X$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Y209" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(Y$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Z209" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(Z$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AA209" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AA$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AB209" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AB$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AC209" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AC$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AD209" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AD$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AE209" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AE$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AF209" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AF$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AG209" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AG$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AH209" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AH$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AI209" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AI$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AJ209" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AJ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AK209" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AK$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AL209" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AL$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AM209" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AM$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AN209" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AN$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AO209" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AO$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AP209" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AP$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AQ209" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AQ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AR209" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AR$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AS209" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$E$32))*Months_In_Year-MONTH(Inputs!$E$32)</f>
+        <f>(AS$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
     </row>
@@ -9542,147 +9313,147 @@
         <v/>
       </c>
       <c r="J211" s="27">
-        <f>(J$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(J$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="K211" s="27">
-        <f>(K$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(K$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="L211" s="27">
-        <f>(L$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(L$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="M211" s="27">
-        <f>(M$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(M$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="N211" s="27">
-        <f>(N$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(N$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="O211" s="27">
-        <f>(O$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(O$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="P211" s="27">
-        <f>(P$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(P$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Q211" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(Q$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="R211" s="27">
-        <f>(R$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(R$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="S211" s="27">
-        <f>(S$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(S$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="T211" s="27">
-        <f>(T$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(T$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="U211" s="27">
-        <f>(U$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(U$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="V211" s="27">
-        <f>(V$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(V$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="W211" s="27">
-        <f>(W$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(W$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="X211" s="27">
-        <f>(X$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(X$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Y211" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(Y$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Z211" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(Z$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AA211" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AA$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AB211" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AB$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AC211" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AC$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AD211" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AD$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AE211" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AE$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AF211" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AF$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AG211" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AG$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AH211" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AH$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AI211" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AI$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ211" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AJ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AK211" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AK$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AL211" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AL$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AM211" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AM$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AN211" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AN$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AO211" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AO$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AP211" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AP$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ211" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AQ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AR211" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AR$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AS211" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$E$33))*Months_In_Year-MONTH(Inputs!$E$33)</f>
+        <f>(AS$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -10178,147 +9949,147 @@
         <v/>
       </c>
       <c r="J215" s="8">
-        <f>($E$62+$E$63)*(J$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(J$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="K215" s="8">
-        <f>($E$62+$E$63)*(K$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(K$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="L215" s="8">
-        <f>($E$62+$E$63)*(L$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(L$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="M215" s="8">
-        <f>($E$62+$E$63)*(M$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(M$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="N215" s="8">
-        <f>($E$62+$E$63)*(N$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(N$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="O215" s="8">
-        <f>($E$62+$E$63)*(O$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(O$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="P215" s="8">
-        <f>($E$62+$E$63)*(P$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(P$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Q215" s="8">
-        <f>($E$62+$E$63)*(Q$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(Q$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="R215" s="8">
-        <f>($E$62+$E$63)*(R$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(R$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="S215" s="8">
-        <f>($E$62+$E$63)*(S$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(S$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="T215" s="8">
-        <f>($E$62+$E$63)*(T$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(T$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="U215" s="8">
-        <f>($E$62+$E$63)*(U$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(U$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="V215" s="8">
-        <f>($E$62+$E$63)*(V$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(V$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="W215" s="8">
-        <f>($E$62+$E$63)*(W$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(W$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="X215" s="8">
-        <f>($E$62+$E$63)*(X$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(X$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Y215" s="8">
-        <f>($E$62+$E$63)*(Y$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(Y$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Z215" s="8">
-        <f>($E$62+$E$63)*(Z$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(Z$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AA215" s="8">
-        <f>($E$62+$E$63)*(AA$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AA$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AB215" s="8">
-        <f>($E$62+$E$63)*(AB$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AB$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AC215" s="8">
-        <f>($E$62+$E$63)*(AC$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AC$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AD215" s="8">
-        <f>($E$62+$E$63)*(AD$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AD$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AE215" s="8">
-        <f>($E$62+$E$63)*(AE$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AE$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AF215" s="8">
-        <f>($E$62+$E$63)*(AF$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AF$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AG215" s="8">
-        <f>($E$62+$E$63)*(AG$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AG$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AH215" s="8">
-        <f>($E$62+$E$63)*(AH$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AH$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AI215" s="8">
-        <f>($E$62+$E$63)*(AI$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AI$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AJ215" s="8">
-        <f>($E$62+$E$63)*(AJ$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AJ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AK215" s="8">
-        <f>($E$62+$E$63)*(AK$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AK$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AL215" s="8">
-        <f>($E$62+$E$63)*(AL$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AL$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AM215" s="8">
-        <f>($E$62+$E$63)*(AM$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AM$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AN215" s="8">
-        <f>($E$62+$E$63)*(AN$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AN$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AO215" s="8">
-        <f>($E$62+$E$63)*(AO$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AO$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AP215" s="8">
-        <f>($E$62+$E$63)*(AP$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AP$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AQ215" s="8">
-        <f>($E$62+$E$63)*(AQ$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AQ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AR215" s="8">
-        <f>($E$62+$E$63)*(AR$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AR$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AS215" s="8">
-        <f>($E$62+$E$63)*(AS$204=YEAR(Inputs!$E$34))</f>
+        <f>($E$62+$E$63)*(AS$204=YEAR(Date_Release))</f>
         <v/>
       </c>
     </row>
@@ -13202,147 +12973,147 @@
         </is>
       </c>
       <c r="J234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-J$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-J$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="K234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-K$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-K$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="L234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-L$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-L$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="M234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-M$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-M$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="N234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-N$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-N$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="O234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-O$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-O$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="P234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-P$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-P$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Q234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-Q$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Q$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="R234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-R$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-R$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="S234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-S$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-S$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="T234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-T$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-T$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="U234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-U$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-U$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="V234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-V$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-V$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="W234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-W$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-W$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="X234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-X$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-X$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Y234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-Y$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Y$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Z234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-Z$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Z$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AA234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AA$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AA$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AB234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AB$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AB$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AC234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AC$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AC$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AD234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AD$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AD$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AE234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AE$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AE$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AF234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AF$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AF$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AG234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AG$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AG$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AH234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AH$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AH$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AI234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AI$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AI$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AJ234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AJ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AJ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AK234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AK$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AK$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AL234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AL$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AL$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AM234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AM$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AM$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AN234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AN$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AN$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AO234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AO$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AO$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AP234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AP$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AP$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AQ234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AQ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AQ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AR234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AR$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AR$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AS234" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$E$33-AS$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AS$205)/Days_In_Year)</f>
         <v/>
       </c>
     </row>
@@ -13740,147 +13511,147 @@
         </is>
       </c>
       <c r="J239" s="27">
-        <f>J$204-YEAR(Inputs!$F$33)</f>
+        <f>J$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="K239" s="27">
-        <f>K$204-YEAR(Inputs!$F$33)</f>
+        <f>K$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="L239" s="27">
-        <f>L$204-YEAR(Inputs!$F$33)</f>
+        <f>L$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="M239" s="27">
-        <f>M$204-YEAR(Inputs!$F$33)</f>
+        <f>M$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="N239" s="27">
-        <f>N$204-YEAR(Inputs!$F$33)</f>
+        <f>N$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="O239" s="27">
-        <f>O$204-YEAR(Inputs!$F$33)</f>
+        <f>O$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="P239" s="27">
-        <f>P$204-YEAR(Inputs!$F$33)</f>
+        <f>P$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Q239" s="27">
-        <f>Q$204-YEAR(Inputs!$F$33)</f>
+        <f>Q$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="R239" s="27">
-        <f>R$204-YEAR(Inputs!$F$33)</f>
+        <f>R$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="S239" s="27">
-        <f>S$204-YEAR(Inputs!$F$33)</f>
+        <f>S$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="T239" s="27">
-        <f>T$204-YEAR(Inputs!$F$33)</f>
+        <f>T$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="U239" s="27">
-        <f>U$204-YEAR(Inputs!$F$33)</f>
+        <f>U$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="V239" s="27">
-        <f>V$204-YEAR(Inputs!$F$33)</f>
+        <f>V$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="W239" s="27">
-        <f>W$204-YEAR(Inputs!$F$33)</f>
+        <f>W$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="X239" s="27">
-        <f>X$204-YEAR(Inputs!$F$33)</f>
+        <f>X$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Y239" s="27">
-        <f>Y$204-YEAR(Inputs!$F$33)</f>
+        <f>Y$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Z239" s="27">
-        <f>Z$204-YEAR(Inputs!$F$33)</f>
+        <f>Z$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AA239" s="27">
-        <f>AA$204-YEAR(Inputs!$F$33)</f>
+        <f>AA$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AB239" s="27">
-        <f>AB$204-YEAR(Inputs!$F$33)</f>
+        <f>AB$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AC239" s="27">
-        <f>AC$204-YEAR(Inputs!$F$33)</f>
+        <f>AC$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AD239" s="27">
-        <f>AD$204-YEAR(Inputs!$F$33)</f>
+        <f>AD$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AE239" s="27">
-        <f>AE$204-YEAR(Inputs!$F$33)</f>
+        <f>AE$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AF239" s="27">
-        <f>AF$204-YEAR(Inputs!$F$33)</f>
+        <f>AF$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AG239" s="27">
-        <f>AG$204-YEAR(Inputs!$F$33)</f>
+        <f>AG$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AH239" s="27">
-        <f>AH$204-YEAR(Inputs!$F$33)</f>
+        <f>AH$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AI239" s="27">
-        <f>AI$204-YEAR(Inputs!$F$33)</f>
+        <f>AI$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ239" s="27">
-        <f>AJ$204-YEAR(Inputs!$F$33)</f>
+        <f>AJ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AK239" s="27">
-        <f>AK$204-YEAR(Inputs!$F$33)</f>
+        <f>AK$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AL239" s="27">
-        <f>AL$204-YEAR(Inputs!$F$33)</f>
+        <f>AL$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AM239" s="27">
-        <f>AM$204-YEAR(Inputs!$F$33)</f>
+        <f>AM$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AN239" s="27">
-        <f>AN$204-YEAR(Inputs!$F$33)</f>
+        <f>AN$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AO239" s="27">
-        <f>AO$204-YEAR(Inputs!$F$33)</f>
+        <f>AO$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AP239" s="27">
-        <f>AP$204-YEAR(Inputs!$F$33)</f>
+        <f>AP$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ239" s="27">
-        <f>AQ$204-YEAR(Inputs!$F$33)</f>
+        <f>AQ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AR239" s="27">
-        <f>AR$204-YEAR(Inputs!$F$33)</f>
+        <f>AR$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AS239" s="27">
-        <f>AS$204-YEAR(Inputs!$F$33)</f>
+        <f>AS$204-YEAR(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -13896,151 +13667,151 @@
         </is>
       </c>
       <c r="F240" s="27">
-        <f>DATEDIF(Inputs!$F$32,Inputs!$F$33,"m")</f>
+        <f>DATEDIF(Date_NTP,Date_COD,"m")</f>
         <v/>
       </c>
       <c r="J240" s="27">
-        <f>(J$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(J$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="K240" s="27">
-        <f>(K$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(K$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="L240" s="27">
-        <f>(L$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(L$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="M240" s="27">
-        <f>(M$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(M$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="N240" s="27">
-        <f>(N$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(N$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="O240" s="27">
-        <f>(O$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(O$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="P240" s="27">
-        <f>(P$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(P$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Q240" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(Q$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="R240" s="27">
-        <f>(R$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(R$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="S240" s="27">
-        <f>(S$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(S$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="T240" s="27">
-        <f>(T$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(T$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="U240" s="27">
-        <f>(U$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(U$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="V240" s="27">
-        <f>(V$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(V$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="W240" s="27">
-        <f>(W$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(W$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="X240" s="27">
-        <f>(X$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(X$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Y240" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(Y$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Z240" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(Z$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AA240" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AA$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AB240" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AB$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AC240" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AC$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AD240" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AD$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AE240" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AE$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AF240" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AF$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AG240" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AG$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AH240" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AH$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AI240" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AI$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AJ240" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AJ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AK240" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AK$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AL240" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AL$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AM240" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AM$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AN240" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AN$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AO240" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AO$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AP240" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AP$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AQ240" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AQ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AR240" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AR$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AS240" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$F$32))*Months_In_Year-MONTH(Inputs!$F$32)</f>
+        <f>(AS$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
     </row>
@@ -14220,147 +13991,147 @@
         <v/>
       </c>
       <c r="J242" s="27">
-        <f>(J$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(J$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="K242" s="27">
-        <f>(K$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(K$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="L242" s="27">
-        <f>(L$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(L$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="M242" s="27">
-        <f>(M$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(M$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="N242" s="27">
-        <f>(N$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(N$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="O242" s="27">
-        <f>(O$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(O$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="P242" s="27">
-        <f>(P$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(P$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Q242" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(Q$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="R242" s="27">
-        <f>(R$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(R$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="S242" s="27">
-        <f>(S$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(S$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="T242" s="27">
-        <f>(T$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(T$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="U242" s="27">
-        <f>(U$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(U$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="V242" s="27">
-        <f>(V$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(V$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="W242" s="27">
-        <f>(W$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(W$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="X242" s="27">
-        <f>(X$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(X$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Y242" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(Y$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Z242" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(Z$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AA242" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AA$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AB242" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AB$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AC242" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AC$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AD242" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AD$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AE242" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AE$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AF242" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AF$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AG242" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AG$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AH242" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AH$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AI242" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AI$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ242" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AJ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AK242" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AK$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AL242" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AL$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AM242" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AM$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AN242" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AN$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AO242" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AO$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AP242" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AP$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ242" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AQ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AR242" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AR$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AS242" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$F$33))*Months_In_Year-MONTH(Inputs!$F$33)</f>
+        <f>(AS$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -14696,147 +14467,147 @@
         <v/>
       </c>
       <c r="J245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=J$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=J$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="K245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=K$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=K$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="L245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=L$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=L$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="M245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=M$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=M$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="N245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=N$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=N$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="O245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=O$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=O$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="P245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=P$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=P$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="Q245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=Q$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Q$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="R245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=R$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=R$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="S245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=S$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=S$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="T245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=T$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=T$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="U245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=U$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=U$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="V245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=V$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=V$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="W245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=W$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=W$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="X245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=X$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=X$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="Y245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=Y$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Y$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="Z245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=Z$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Z$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AA245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AA$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AA$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AB245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AB$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AB$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AC245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AC$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AC$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AD245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AD$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AD$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AE245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AE$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AE$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AF245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AF$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AF$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AG245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AG$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AG$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AH245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AH$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AH$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AI245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AI$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AI$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AJ245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AJ$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AJ$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AK245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AK$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AK$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AL245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AL$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AL$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AM245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AM$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AM$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AN245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AN$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AN$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AO245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AO$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AO$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AP245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AP$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AP$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AQ245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AQ$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AQ$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AR245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AR$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AR$204)*$F$190:$F$197)</f>
         <v/>
       </c>
       <c r="AS245" s="8">
-        <f>SUMPRODUCT((YEAR($K$190:$K$197)=AS$204)*$F$190:$F$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AS$204)*$F$190:$F$197)</f>
         <v/>
       </c>
     </row>
@@ -14856,147 +14627,147 @@
         <v/>
       </c>
       <c r="J246" s="8">
-        <f>($F$62+$F$63)*(J$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(J$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="K246" s="8">
-        <f>($F$62+$F$63)*(K$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(K$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="L246" s="8">
-        <f>($F$62+$F$63)*(L$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(L$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="M246" s="8">
-        <f>($F$62+$F$63)*(M$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(M$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="N246" s="8">
-        <f>($F$62+$F$63)*(N$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(N$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="O246" s="8">
-        <f>($F$62+$F$63)*(O$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(O$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="P246" s="8">
-        <f>($F$62+$F$63)*(P$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(P$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Q246" s="8">
-        <f>($F$62+$F$63)*(Q$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(Q$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="R246" s="8">
-        <f>($F$62+$F$63)*(R$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(R$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="S246" s="8">
-        <f>($F$62+$F$63)*(S$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(S$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="T246" s="8">
-        <f>($F$62+$F$63)*(T$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(T$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="U246" s="8">
-        <f>($F$62+$F$63)*(U$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(U$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="V246" s="8">
-        <f>($F$62+$F$63)*(V$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(V$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="W246" s="8">
-        <f>($F$62+$F$63)*(W$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(W$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="X246" s="8">
-        <f>($F$62+$F$63)*(X$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(X$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Y246" s="8">
-        <f>($F$62+$F$63)*(Y$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(Y$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Z246" s="8">
-        <f>($F$62+$F$63)*(Z$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(Z$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AA246" s="8">
-        <f>($F$62+$F$63)*(AA$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AA$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AB246" s="8">
-        <f>($F$62+$F$63)*(AB$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AB$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AC246" s="8">
-        <f>($F$62+$F$63)*(AC$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AC$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AD246" s="8">
-        <f>($F$62+$F$63)*(AD$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AD$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AE246" s="8">
-        <f>($F$62+$F$63)*(AE$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AE$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AF246" s="8">
-        <f>($F$62+$F$63)*(AF$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AF$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AG246" s="8">
-        <f>($F$62+$F$63)*(AG$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AG$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AH246" s="8">
-        <f>($F$62+$F$63)*(AH$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AH$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AI246" s="8">
-        <f>($F$62+$F$63)*(AI$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AI$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AJ246" s="8">
-        <f>($F$62+$F$63)*(AJ$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AJ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AK246" s="8">
-        <f>($F$62+$F$63)*(AK$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AK$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AL246" s="8">
-        <f>($F$62+$F$63)*(AL$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AL$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AM246" s="8">
-        <f>($F$62+$F$63)*(AM$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AM$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AN246" s="8">
-        <f>($F$62+$F$63)*(AN$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AN$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AO246" s="8">
-        <f>($F$62+$F$63)*(AO$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AO$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AP246" s="8">
-        <f>($F$62+$F$63)*(AP$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AP$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AQ246" s="8">
-        <f>($F$62+$F$63)*(AQ$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AQ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AR246" s="8">
-        <f>($F$62+$F$63)*(AR$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AR$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AS246" s="8">
-        <f>($F$62+$F$63)*(AS$204=YEAR(Inputs!$F$34))</f>
+        <f>($F$62+$F$63)*(AS$204=YEAR(Date_Release))</f>
         <v/>
       </c>
     </row>
@@ -17880,147 +17651,147 @@
         </is>
       </c>
       <c r="J265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-J$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-J$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="K265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-K$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-K$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="L265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-L$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-L$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="M265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-M$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-M$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="N265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-N$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-N$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="O265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-O$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-O$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="P265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-P$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-P$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Q265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-Q$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Q$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="R265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-R$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-R$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="S265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-S$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-S$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="T265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-T$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-T$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="U265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-U$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-U$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="V265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-V$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-V$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="W265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-W$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-W$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="X265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-X$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-X$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Y265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-Y$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Y$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Z265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-Z$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Z$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AA265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AA$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AA$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AB265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AB$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AB$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AC265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AC$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AC$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AD265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AD$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AD$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AE265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AE$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AE$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AF265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AF$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AF$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AG265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AG$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AG$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AH265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AH$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AH$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AI265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AI$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AI$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AJ265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AJ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AJ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AK265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AK$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AK$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AL265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AL$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AL$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AM265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AM$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AM$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AN265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AN$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AN$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AO265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AO$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AO$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AP265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AP$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AP$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AQ265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AQ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AQ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AR265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AR$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AR$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AS265" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$F$33-AS$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AS$205)/Days_In_Year)</f>
         <v/>
       </c>
     </row>
@@ -18418,147 +18189,147 @@
         </is>
       </c>
       <c r="J270" s="27">
-        <f>J$204-YEAR(Inputs!$G$33)</f>
+        <f>J$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="K270" s="27">
-        <f>K$204-YEAR(Inputs!$G$33)</f>
+        <f>K$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="L270" s="27">
-        <f>L$204-YEAR(Inputs!$G$33)</f>
+        <f>L$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="M270" s="27">
-        <f>M$204-YEAR(Inputs!$G$33)</f>
+        <f>M$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="N270" s="27">
-        <f>N$204-YEAR(Inputs!$G$33)</f>
+        <f>N$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="O270" s="27">
-        <f>O$204-YEAR(Inputs!$G$33)</f>
+        <f>O$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="P270" s="27">
-        <f>P$204-YEAR(Inputs!$G$33)</f>
+        <f>P$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Q270" s="27">
-        <f>Q$204-YEAR(Inputs!$G$33)</f>
+        <f>Q$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="R270" s="27">
-        <f>R$204-YEAR(Inputs!$G$33)</f>
+        <f>R$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="S270" s="27">
-        <f>S$204-YEAR(Inputs!$G$33)</f>
+        <f>S$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="T270" s="27">
-        <f>T$204-YEAR(Inputs!$G$33)</f>
+        <f>T$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="U270" s="27">
-        <f>U$204-YEAR(Inputs!$G$33)</f>
+        <f>U$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="V270" s="27">
-        <f>V$204-YEAR(Inputs!$G$33)</f>
+        <f>V$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="W270" s="27">
-        <f>W$204-YEAR(Inputs!$G$33)</f>
+        <f>W$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="X270" s="27">
-        <f>X$204-YEAR(Inputs!$G$33)</f>
+        <f>X$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Y270" s="27">
-        <f>Y$204-YEAR(Inputs!$G$33)</f>
+        <f>Y$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="Z270" s="27">
-        <f>Z$204-YEAR(Inputs!$G$33)</f>
+        <f>Z$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AA270" s="27">
-        <f>AA$204-YEAR(Inputs!$G$33)</f>
+        <f>AA$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AB270" s="27">
-        <f>AB$204-YEAR(Inputs!$G$33)</f>
+        <f>AB$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AC270" s="27">
-        <f>AC$204-YEAR(Inputs!$G$33)</f>
+        <f>AC$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AD270" s="27">
-        <f>AD$204-YEAR(Inputs!$G$33)</f>
+        <f>AD$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AE270" s="27">
-        <f>AE$204-YEAR(Inputs!$G$33)</f>
+        <f>AE$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AF270" s="27">
-        <f>AF$204-YEAR(Inputs!$G$33)</f>
+        <f>AF$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AG270" s="27">
-        <f>AG$204-YEAR(Inputs!$G$33)</f>
+        <f>AG$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AH270" s="27">
-        <f>AH$204-YEAR(Inputs!$G$33)</f>
+        <f>AH$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AI270" s="27">
-        <f>AI$204-YEAR(Inputs!$G$33)</f>
+        <f>AI$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ270" s="27">
-        <f>AJ$204-YEAR(Inputs!$G$33)</f>
+        <f>AJ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AK270" s="27">
-        <f>AK$204-YEAR(Inputs!$G$33)</f>
+        <f>AK$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AL270" s="27">
-        <f>AL$204-YEAR(Inputs!$G$33)</f>
+        <f>AL$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AM270" s="27">
-        <f>AM$204-YEAR(Inputs!$G$33)</f>
+        <f>AM$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AN270" s="27">
-        <f>AN$204-YEAR(Inputs!$G$33)</f>
+        <f>AN$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AO270" s="27">
-        <f>AO$204-YEAR(Inputs!$G$33)</f>
+        <f>AO$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AP270" s="27">
-        <f>AP$204-YEAR(Inputs!$G$33)</f>
+        <f>AP$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ270" s="27">
-        <f>AQ$204-YEAR(Inputs!$G$33)</f>
+        <f>AQ$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AR270" s="27">
-        <f>AR$204-YEAR(Inputs!$G$33)</f>
+        <f>AR$204-YEAR(Date_COD)</f>
         <v/>
       </c>
       <c r="AS270" s="27">
-        <f>AS$204-YEAR(Inputs!$G$33)</f>
+        <f>AS$204-YEAR(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -18574,151 +18345,151 @@
         </is>
       </c>
       <c r="G271" s="27">
-        <f>DATEDIF(Inputs!$G$32,Inputs!$G$33,"m")</f>
+        <f>DATEDIF(Date_NTP,Date_COD,"m")</f>
         <v/>
       </c>
       <c r="J271" s="27">
-        <f>(J$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(J$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="K271" s="27">
-        <f>(K$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(K$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="L271" s="27">
-        <f>(L$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(L$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="M271" s="27">
-        <f>(M$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(M$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="N271" s="27">
-        <f>(N$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(N$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="O271" s="27">
-        <f>(O$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(O$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="P271" s="27">
-        <f>(P$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(P$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Q271" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(Q$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="R271" s="27">
-        <f>(R$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(R$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="S271" s="27">
-        <f>(S$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(S$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="T271" s="27">
-        <f>(T$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(T$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="U271" s="27">
-        <f>(U$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(U$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="V271" s="27">
-        <f>(V$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(V$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="W271" s="27">
-        <f>(W$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(W$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="X271" s="27">
-        <f>(X$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(X$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Y271" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(Y$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="Z271" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(Z$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AA271" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AA$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AB271" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AB$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AC271" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AC$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AD271" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AD$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AE271" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AE$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AF271" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AF$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AG271" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AG$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AH271" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AH$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AI271" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AI$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AJ271" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AJ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AK271" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AK$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AL271" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AL$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AM271" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AM$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AN271" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AN$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AO271" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AO$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AP271" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AP$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AQ271" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AQ$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AR271" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AR$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
       <c r="AS271" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$G$32))*Months_In_Year-MONTH(Inputs!$G$32)</f>
+        <f>(AS$204+1-YEAR(Date_NTP))*Months_In_Year-MONTH(Date_NTP)</f>
         <v/>
       </c>
     </row>
@@ -18898,147 +18669,147 @@
         <v/>
       </c>
       <c r="J273" s="27">
-        <f>(J$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(J$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="K273" s="27">
-        <f>(K$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(K$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="L273" s="27">
-        <f>(L$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(L$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="M273" s="27">
-        <f>(M$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(M$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="N273" s="27">
-        <f>(N$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(N$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="O273" s="27">
-        <f>(O$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(O$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="P273" s="27">
-        <f>(P$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(P$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Q273" s="27">
-        <f>(Q$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(Q$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="R273" s="27">
-        <f>(R$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(R$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="S273" s="27">
-        <f>(S$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(S$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="T273" s="27">
-        <f>(T$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(T$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="U273" s="27">
-        <f>(U$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(U$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="V273" s="27">
-        <f>(V$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(V$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="W273" s="27">
-        <f>(W$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(W$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="X273" s="27">
-        <f>(X$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(X$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Y273" s="27">
-        <f>(Y$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(Y$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="Z273" s="27">
-        <f>(Z$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(Z$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AA273" s="27">
-        <f>(AA$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AA$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AB273" s="27">
-        <f>(AB$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AB$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AC273" s="27">
-        <f>(AC$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AC$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AD273" s="27">
-        <f>(AD$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AD$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AE273" s="27">
-        <f>(AE$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AE$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AF273" s="27">
-        <f>(AF$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AF$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AG273" s="27">
-        <f>(AG$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AG$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AH273" s="27">
-        <f>(AH$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AH$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AI273" s="27">
-        <f>(AI$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AI$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AJ273" s="27">
-        <f>(AJ$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AJ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AK273" s="27">
-        <f>(AK$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AK$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AL273" s="27">
-        <f>(AL$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AL$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AM273" s="27">
-        <f>(AM$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AM$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AN273" s="27">
-        <f>(AN$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AN$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AO273" s="27">
-        <f>(AO$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AO$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AP273" s="27">
-        <f>(AP$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AP$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AQ273" s="27">
-        <f>(AQ$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AQ$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AR273" s="27">
-        <f>(AR$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AR$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
       <c r="AS273" s="27">
-        <f>(AS$204+1-YEAR(Inputs!$G$33))*Months_In_Year-MONTH(Inputs!$G$33)</f>
+        <f>(AS$204+1-YEAR(Date_COD))*Months_In_Year-MONTH(Date_COD)</f>
         <v/>
       </c>
     </row>
@@ -19374,147 +19145,147 @@
         <v/>
       </c>
       <c r="J276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=J$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=J$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="K276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=K$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=K$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="L276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=L$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=L$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="M276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=M$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=M$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="N276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=N$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=N$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="O276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=O$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=O$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="P276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=P$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=P$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="Q276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=Q$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Q$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="R276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=R$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=R$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="S276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=S$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=S$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="T276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=T$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=T$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="U276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=U$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=U$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="V276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=V$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=V$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="W276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=W$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=W$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="X276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=X$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=X$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="Y276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=Y$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Y$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="Z276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=Z$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=Z$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AA276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AA$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AA$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AB276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AB$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AB$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AC276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AC$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AC$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AD276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AD$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AD$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AE276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AE$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AE$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AF276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AF$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AF$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AG276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AG$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AG$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AH276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AH$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AH$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AI276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AI$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AI$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AJ276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AJ$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AJ$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AK276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AK$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AK$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AL276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AL$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AL$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AM276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AM$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AM$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AN276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AN$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AN$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AO276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AO$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AO$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AP276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AP$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AP$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AQ276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AQ$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AQ$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AR276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AR$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AR$204)*$G$190:$G$197)</f>
         <v/>
       </c>
       <c r="AS276" s="8">
-        <f>SUMPRODUCT((YEAR($L$190:$L$197)=AS$204)*$G$190:$G$197)</f>
+        <f>SUMPRODUCT((YEAR($J$190:$J$197)=AS$204)*$G$190:$G$197)</f>
         <v/>
       </c>
     </row>
@@ -19534,147 +19305,147 @@
         <v/>
       </c>
       <c r="J277" s="8">
-        <f>($G$62+$G$63)*(J$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(J$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="K277" s="8">
-        <f>($G$62+$G$63)*(K$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(K$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="L277" s="8">
-        <f>($G$62+$G$63)*(L$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(L$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="M277" s="8">
-        <f>($G$62+$G$63)*(M$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(M$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="N277" s="8">
-        <f>($G$62+$G$63)*(N$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(N$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="O277" s="8">
-        <f>($G$62+$G$63)*(O$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(O$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="P277" s="8">
-        <f>($G$62+$G$63)*(P$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(P$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Q277" s="8">
-        <f>($G$62+$G$63)*(Q$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(Q$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="R277" s="8">
-        <f>($G$62+$G$63)*(R$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(R$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="S277" s="8">
-        <f>($G$62+$G$63)*(S$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(S$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="T277" s="8">
-        <f>($G$62+$G$63)*(T$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(T$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="U277" s="8">
-        <f>($G$62+$G$63)*(U$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(U$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="V277" s="8">
-        <f>($G$62+$G$63)*(V$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(V$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="W277" s="8">
-        <f>($G$62+$G$63)*(W$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(W$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="X277" s="8">
-        <f>($G$62+$G$63)*(X$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(X$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Y277" s="8">
-        <f>($G$62+$G$63)*(Y$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(Y$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="Z277" s="8">
-        <f>($G$62+$G$63)*(Z$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(Z$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AA277" s="8">
-        <f>($G$62+$G$63)*(AA$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AA$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AB277" s="8">
-        <f>($G$62+$G$63)*(AB$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AB$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AC277" s="8">
-        <f>($G$62+$G$63)*(AC$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AC$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AD277" s="8">
-        <f>($G$62+$G$63)*(AD$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AD$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AE277" s="8">
-        <f>($G$62+$G$63)*(AE$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AE$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AF277" s="8">
-        <f>($G$62+$G$63)*(AF$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AF$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AG277" s="8">
-        <f>($G$62+$G$63)*(AG$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AG$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AH277" s="8">
-        <f>($G$62+$G$63)*(AH$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AH$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AI277" s="8">
-        <f>($G$62+$G$63)*(AI$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AI$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AJ277" s="8">
-        <f>($G$62+$G$63)*(AJ$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AJ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AK277" s="8">
-        <f>($G$62+$G$63)*(AK$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AK$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AL277" s="8">
-        <f>($G$62+$G$63)*(AL$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AL$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AM277" s="8">
-        <f>($G$62+$G$63)*(AM$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AM$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AN277" s="8">
-        <f>($G$62+$G$63)*(AN$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AN$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AO277" s="8">
-        <f>($G$62+$G$63)*(AO$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AO$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AP277" s="8">
-        <f>($G$62+$G$63)*(AP$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AP$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AQ277" s="8">
-        <f>($G$62+$G$63)*(AQ$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AQ$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AR277" s="8">
-        <f>($G$62+$G$63)*(AR$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AR$204=YEAR(Date_Release))</f>
         <v/>
       </c>
       <c r="AS277" s="8">
-        <f>($G$62+$G$63)*(AS$204=YEAR(Inputs!$G$34))</f>
+        <f>($G$62+$G$63)*(AS$204=YEAR(Date_Release))</f>
         <v/>
       </c>
     </row>
@@ -22558,147 +22329,147 @@
         </is>
       </c>
       <c r="J296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-J$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-J$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="K296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-K$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-K$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="L296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-L$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-L$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="M296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-M$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-M$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="N296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-N$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-N$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="O296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-O$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-O$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="P296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-P$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-P$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Q296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-Q$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Q$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="R296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-R$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-R$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="S296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-S$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-S$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="T296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-T$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-T$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="U296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-U$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-U$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="V296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-V$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-V$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="W296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-W$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-W$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="X296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-X$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-X$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Y296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-Y$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Y$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="Z296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-Z$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-Z$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AA296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AA$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AA$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AB296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AB$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AB$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AC296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AC$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AC$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AD296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AD$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AD$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AE296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AE$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AE$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AF296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AF$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AF$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AG296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AG$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AG$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AH296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AH$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AH$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AI296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AI$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AI$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AJ296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AJ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AJ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AK296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AK$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AK$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AL296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AL$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AL$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AM296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AM$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AM$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AN296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AN$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AN$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AO296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AO$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AO$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AP296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AP$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AP$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AQ296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AQ$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AQ$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AR296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AR$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AR$205)/Days_In_Year)</f>
         <v/>
       </c>
       <c r="AS296" s="30">
-        <f>(1+Discount_Rate)^((Inputs!$G$33-AS$205)/Days_In_Year)</f>
+        <f>(1+Discount_Rate)^((Date_COD-AS$205)/Days_In_Year)</f>
         <v/>
       </c>
     </row>
@@ -23190,11 +22961,11 @@
         <v/>
       </c>
       <c r="F306" s="29">
-        <f>SUMPRODUCT(--(YEAR(K191:K197)&gt;=YEAR(F153)))</f>
+        <f>SUMPRODUCT(--(YEAR(J191:J197)&gt;=YEAR(F153)))</f>
         <v/>
       </c>
       <c r="G306" s="29">
-        <f>SUMPRODUCT(--(YEAR(L191:L197)&gt;=YEAR(G153)))</f>
+        <f>SUMPRODUCT(--(YEAR(J191:J197)&gt;=YEAR(G153)))</f>
         <v/>
       </c>
       <c r="H306" s="29">
@@ -23928,35 +23699,21 @@
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Signing fee and DD paid</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="E26" s="33" t="n">
-        <v>46234</v>
-      </c>
-      <c r="F26" s="33" t="n">
-        <v>46234</v>
-      </c>
-      <c r="G26" s="33" t="n">
-        <v>46234</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Bora Inputs E27; Bid_Cash E34</t>
-        </is>
-      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Key dates (all projects; value in column E)</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="21" t="n"/>
     </row>
     <row r="27">
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Bid submission: fee paid, bid security posted</t>
+          <t>Signing fee and DD paid</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -23965,24 +23722,18 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>46325</v>
-      </c>
-      <c r="F27" s="33" t="n">
-        <v>46325</v>
-      </c>
-      <c r="G27" s="33" t="n">
-        <v>46325</v>
+        <v>46234</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E95; Bid_Cash E35</t>
+          <t>Bid_Cash E34</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Performance security posted</t>
+          <t>Bid submission: fee paid, bid security posted</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -23991,24 +23742,18 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
-        <v>46386</v>
-      </c>
-      <c r="F28" s="33" t="n">
-        <v>46402</v>
-      </c>
-      <c r="G28" s="33" t="n">
-        <v>46402</v>
+        <v>46325</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Bora Deposits K10 (E96 + 17 d); Bid_Cash E36</t>
+          <t>Bid_Cash E35</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>TSO security paid</t>
+          <t>Performance security posted (bid security credited)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -24017,24 +23762,18 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>46386</v>
-      </c>
-      <c r="F29" s="33" t="n">
         <v>46402</v>
       </c>
-      <c r="G29" s="33" t="n">
-        <v>46402</v>
-      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E97; Bid_Cash E37</t>
+          <t>Bid_Cash E36</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Connection agreement (HCSSZ): fees paid</t>
+          <t>TSO security paid</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -24043,24 +23782,18 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
-        <v>47027</v>
-      </c>
-      <c r="F30" s="33" t="n">
-        <v>47027</v>
-      </c>
-      <c r="G30" s="33" t="n">
-        <v>47027</v>
+        <v>46402</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E99; Bid_Cash E39</t>
+          <t>Bid_Cash E37</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Devex average payment date</t>
+          <t>Devex average payment date (spent continuously)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -24069,24 +23802,18 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>46768</v>
-      </c>
-      <c r="F31" s="33" t="n">
         <v>46752</v>
       </c>
-      <c r="G31" s="33" t="n">
-        <v>46752</v>
-      </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Bora Devex_FEP, amount-weighted; Bid_Cash 'continuous'</t>
+          <t>Bid_Cash H77 'continuous'; SPEC §21.1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Notice to proceed</t>
+          <t>Connection agreement (HCSSZ): fees paid</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -24095,24 +23822,18 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
-        <v>47299</v>
-      </c>
-      <c r="F32" s="33" t="n">
-        <v>47299</v>
-      </c>
-      <c r="G32" s="33" t="n">
-        <v>47299</v>
+        <v>47027</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E154; Bid_Cash E40</t>
+          <t>Bid_Cash E39</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Notice to proceed</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -24121,24 +23842,18 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>48029</v>
-      </c>
-      <c r="F33" s="33" t="n">
-        <v>48029</v>
-      </c>
-      <c r="G33" s="33" t="n">
-        <v>48029</v>
+        <v>47299</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E155; Bid_Cash E41</t>
+          <t>Bid_Cash E40</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Performance security released</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -24147,24 +23862,18 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
-        <v>48669</v>
-      </c>
-      <c r="F34" s="33" t="n">
-        <v>48669</v>
-      </c>
-      <c r="G34" s="33" t="n">
-        <v>48669</v>
+        <v>48029</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Bid_Cash E42 (Kiírás XII.13, estimate)</t>
+          <t>Bid_Cash E41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>DSA accrual start</t>
+          <t>Performance security released</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -24173,17 +23882,11 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>46321</v>
-      </c>
-      <c r="F35" s="33" t="n">
-        <v>46234</v>
-      </c>
-      <c r="G35" s="33" t="n">
-        <v>46234</v>
+        <v>48669</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Bora Inputs E70; others: signing (DSA off)</t>
+          <t>Bid_Cash E42 (estimate)</t>
         </is>
       </c>
     </row>
@@ -24322,7 +24025,7 @@
     <row r="43">
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Developer success fee (on committed MW, 30/360)</t>
+          <t>Developer success fee (on committed MW, signing to sale, 30/360)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">

</xml_diff>